<commit_message>
chore: update NEXUS prices (drug store 4125, pharmacy 4389)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/templates/Hikma orders.xlsx
+++ b/backend/templates/Hikma orders.xlsx
@@ -793,10 +793,10 @@
         <v>9</v>
       </c>
       <c r="B7" s="12">
-        <v>6187</v>
+        <v>4125</v>
       </c>
       <c r="C7" s="12">
-        <v>6583</v>
+        <v>4389</v>
       </c>
       <c r="D7" s="10"/>
       <c r="E7" s="10"/>

</xml_diff>